<commit_message>
Rebuild Excel model from the current perfect-competition-spec.md
Regenerated model.xlsx from scratch against the spec as it stands now
(FARMER_RATE = FARMER_SALARY / FARMER_FULL_HRS, the case's per-crop
compounding labor formula, all other sections unchanged since the last
build). Same five sheets, same formulas, same recommendation:
N_TEMP=3, 10/19/28 beds, profit $16,586.

Verified with the Python `formulas` engine (LibreOffice and Excel
automation remain unavailable in this environment): 769 cells, zero
errors, every hand-checked value — FARMER_RATE, the published tomato
bed-10 check figures, all five N_TEMP profit figures, the recommended
mix, and the P&L reconciliation — matches ground truth exactly, same
as the previous build.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -79,7 +79,7 @@
     <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -128,16 +128,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00008000"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -184,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -228,11 +220,11 @@
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -241,12 +233,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -648,8 +634,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -804,7 +790,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Case scenario, header line. This is her actual field-time contribution to LABOR_SUPPLY — half her working time.</t>
+          <t>Case scenario, header line. Her actual field-time contribution to LABOR_SUPPLY — half her working time.</t>
         </is>
       </c>
     </row>
@@ -1103,15 +1089,16 @@
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>PRICE_c is revenue per bed — the case has already collapsed price per unit and yield per bed into one figure, so yield is not modeled separately and per-bed revenue does not decline with scale. Every nonlinearity in this model lives in labor hours (see the Labor sheet).</t>
+          <t>PRICE_c is revenue per bed — the case has already collapsed price per unit and yield per bed into one figure, so yield is not modeled separately and per-bed revenue does not decline with scale. Every nonlinearity in this model lives in labor hours (see the Labor sheet). Diminishing returns compound on the whole crop, not incrementally per bed: every one of the q beds planted of a crop is charged the same (1+DIM)^q multiplier — see Labor sheet.</t>
         </is>
       </c>
     </row>
     <row r="29"/>
     <row r="30"/>
+    <row r="31"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A28:F30"/>
+    <mergeCell ref="A28:F31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1125,7 +1112,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E90"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1144,7 +1131,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>LABOR_HRS_c(q) = SEASON_HRS_PER_BED_c x q x (1+DIM_c)^q   |   MARGINAL_LABOR_HRS_c(q) = LABOR_HRS_c(q) - LABOR_HRS_c(q-1)   |   MC_c(q) = MARGINAL_LABOR_HRS_c(q) x TEMP_RATE + FERT_c</t>
+          <t>LABOR_HRS_c(q) = SEASON_HRS_PER_BED_c x q x (1+DIM_c)^q   |   MARGINAL_LABOR_HRS_c(q) = SEASON_HRS_PER_BED_c x (1+DIM_c)^(q-1) x (1+q x DIM_c)   |   MC_c(q) = MARGINAL_LABOR_HRS_c(q) x TEMP_RATE + FERT_c</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2819,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -3419,7 +3406,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -3688,8 +3675,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
@@ -3786,7 +3773,7 @@
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
-          <t>See Audit finding 1: this test is only meaningful when the crop stopped for its own MC=PRICE reason, not for lack of shared labor.</t>
+          <t>See Audit finding 2: this test is only meaningful when the crop stopped for its own MC=PRICE reason, not for lack of shared labor.</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3792,7 @@
       </c>
       <c r="D8" s="40" t="inlineStr">
         <is>
-          <t>Expected to read FAIL here as literally worded — carrots stop because labor runs out, not because bed 20 is unprofitable. See Audit finding 1.</t>
+          <t>Expected to read FAIL here as literally worded — carrots stop because labor runs out, not because the next bed is unprofitable. See Audit finding 2.</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3811,7 @@
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
-          <t>Expected to read FAIL here as literally worded, for the same reason as Carrots. See Audit finding 1.</t>
+          <t>Expected to read FAIL here as literally worded, for the same reason as Carrots. See Audit finding 2.</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3916,7 @@
       </c>
       <c r="D16" s="40" t="inlineStr">
         <is>
-          <t>See P&amp;L sheet, bottom row.</t>
+          <t>See P&amp;L sheet.</t>
         </is>
       </c>
     </row>
@@ -3995,52 +3982,16 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Added after the build, per the spec's template.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="42" t="inlineStr">
-        <is>
-          <t>1. Validation rule 4 (price-taker test) is mis-specified for a labor-constrained crop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="43" t="inlineStr">
-        <is>
-          <t>Checked: whether rule 4, as literally worded in the spec, holds for every crop at the recommended mix (N_TEMP=3, 10/19/28 beds). Found: it fails for Carrots and Mesclun. Both stop short of their own MC=PRICE point — Carrots at 19 beds when bed 20 is still individually profitable (MC≈$1,689 &lt; PRICE $2,094), Mesclun at 28 when bed 29 is too — because there are only 10.25 labor hours of slack left and neither crop's next bed fits in it (Carrot bed 20 alone needs 71.9 hours). The rule's premise ("LABOR_SLACK &gt; 0") is satisfied even though labor is what actually stopped them, so the test fires incorrectly. What I did: implemented the check exactly as specified (so the failure is visible, not hidden) and flagged the rule for revision — it should read something like "...MC_c(Q_c+1) &gt;= PRICE_c OR MARGINAL_LABOR_HRS_c(Q_c+1) &gt; LABOR_SLACK".</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="30">
-      <c r="A30" s="42" t="inlineStr">
-        <is>
-          <t>2. A $/hour greedy heuristic does not find the true optimum — exhaustive search was necessary.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="90" customHeight="1">
-      <c r="A31" s="43" t="inlineStr">
-        <is>
-          <t>Checked: whether ranking every candidate bed (all three crops, all bed counts) by contribution per labor hour and taking them greedily until the budget runs out reproduces the optimum. Found: it does not, at any N_TEMP. At N_TEMP=3 the greedy rule lands on 9/20/30 beds for $13,960 profit; exhaustive integer search finds 10/19/28 for $16,586 — nearly $2,600 better, using MORE labor hours, not fewer. Greedy locks in early high-density beds (mesclun, whose 1.25% diminishing-returns rate makes it look cheap) and leaves no room for a combination that is better in total even though no single swap looks like an improvement from where greedy stands. What I did: solved by exhaustive integer search (21x21x31 combinations per N_TEMP) instead, and set up the Optimize sheet so the same search is reproducible in Excel via Solver (Evolutionary engine — GRG Nonlinear should not be trusted on this labor formula, and a greedy/manual ranking should not be trusted at all).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>See the spec's own Audit findings section for the full narrative (FARMER_RATE bug, the price-taker test gap for Carrots/Mesclun, why a $/hour greedy ranking fails here, and the LibreOffice/Excel-automation substitution used to verify this workbook).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A31:D34"/>
-    <mergeCell ref="A25:D28"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A30:D30"/>
+  <mergeCells count="1">
+    <mergeCell ref="A22:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>